<commit_message>
Integra integracao Sances com agendamentos estoque e IA
</commit_message>
<xml_diff>
--- a/templates/data/disparo_atacado.xlsx
+++ b/templates/data/disparo_atacado.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U204"/>
+  <dimension ref="A1:U243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17208,6 +17208,3555 @@
         </is>
       </c>
     </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Atacadão Moto Peças</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Oficina mecânica de motos</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>(99) 98526-2063</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>5599985262063</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr"/>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:17</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr"/>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:17</t>
+        </is>
+      </c>
+      <c r="M205" t="inlineStr"/>
+      <c r="N205" t="inlineStr"/>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P205" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q205" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R205" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S205" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T205" t="inlineStr">
+        <is>
+          <t>8A9BB54EB1B3F52A4C1E</t>
+        </is>
+      </c>
+      <c r="U205" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Cortez Motos - Rua Ceará</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Loja de peças para motocicletas</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>(99) 3524-5888</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>559935245888</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr"/>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:18</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr"/>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:18</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr"/>
+      <c r="N206" t="inlineStr"/>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P206" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q206" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R206" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S206" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T206" t="inlineStr">
+        <is>
+          <t>3EB0F9E0423C6604D8D887</t>
+        </is>
+      </c>
+      <c r="U206" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Atacadão Moto Peças 2</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Loja de peças para motocicletas</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>(99) 98528-1303</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>5599985281303</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr"/>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:20</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K207" t="inlineStr"/>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:20</t>
+        </is>
+      </c>
+      <c r="M207" t="inlineStr"/>
+      <c r="N207" t="inlineStr"/>
+      <c r="O207" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P207" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q207" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R207" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S207" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T207" t="inlineStr">
+        <is>
+          <t>3EB0FABE74F8CA6CEF2F1F</t>
+        </is>
+      </c>
+      <c r="U207" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Motor peças motosserras em Imperatriz - roçadeiras em Imperatriz -motores estacionário em Imperatriz</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Fornecedor de equipamentos agrícolas</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>(99) 3525-7772</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>559935257772</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr"/>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:21</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr"/>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:21</t>
+        </is>
+      </c>
+      <c r="M208" t="inlineStr"/>
+      <c r="N208" t="inlineStr"/>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P208" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q208" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R208" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S208" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T208" t="inlineStr">
+        <is>
+          <t>3EB0CCF932094BE85DAC44</t>
+        </is>
+      </c>
+      <c r="U208" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Tony Moto Peças</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Loja de autopeças</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>(99) 98242-9668</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>5599982429668</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr"/>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:23</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr"/>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:23</t>
+        </is>
+      </c>
+      <c r="M209" t="inlineStr"/>
+      <c r="N209" t="inlineStr"/>
+      <c r="O209" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P209" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q209" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R209" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S209" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T209" t="inlineStr">
+        <is>
+          <t>3EB0C9788463329C7C080C</t>
+        </is>
+      </c>
+      <c r="U209" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Luso Motos Comércio e Distribuição Ltda</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Loja de peças para motocicletas</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>(99) 3524-4505</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>559935244505</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr"/>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:24</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr"/>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:24</t>
+        </is>
+      </c>
+      <c r="M210" t="inlineStr"/>
+      <c r="N210" t="inlineStr"/>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P210" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q210" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R210" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S210" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T210" t="inlineStr">
+        <is>
+          <t>3EB00B1E417FBE8E33D212</t>
+        </is>
+      </c>
+      <c r="U210" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>STRELA MOTO PEÇAS - Atacado e Varejo</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Oficina mecânica de motos</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>(99) 98433-1186</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>5599984331186</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr"/>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:26</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K211" t="inlineStr"/>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:26</t>
+        </is>
+      </c>
+      <c r="M211" t="inlineStr"/>
+      <c r="N211" t="inlineStr"/>
+      <c r="O211" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P211" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q211" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R211" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S211" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T211" t="inlineStr">
+        <is>
+          <t>3EB06F060AD7776C02388F</t>
+        </is>
+      </c>
+      <c r="U211" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>KSS MOTOS CEARÁ ITZ</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Loja de motocicletas</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>(99) 98476-2923</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>5599984762923</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr"/>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:27</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K212" t="inlineStr"/>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:27</t>
+        </is>
+      </c>
+      <c r="M212" t="inlineStr"/>
+      <c r="N212" t="inlineStr"/>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P212" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q212" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R212" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S212" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T212" t="inlineStr">
+        <is>
+          <t>3EB0B2C3BB40400D02488C</t>
+        </is>
+      </c>
+      <c r="U212" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Damásio Motopeças Imperatriz</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Loja de peças para motocicletas</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>(86) 3131-8320</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>558631318320</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr"/>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:29</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K213" t="inlineStr"/>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:29</t>
+        </is>
+      </c>
+      <c r="M213" t="inlineStr"/>
+      <c r="N213" t="inlineStr"/>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P213" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q213" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R213" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S213" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T213" t="inlineStr">
+        <is>
+          <t>3EB0AC7E44C4339432D0DB</t>
+        </is>
+      </c>
+      <c r="U213" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>s.a moto pecas</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Loja de peças para motocicletas</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>(99) 98543-3274</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>5599985433274</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr"/>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:30</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr"/>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:30</t>
+        </is>
+      </c>
+      <c r="M214" t="inlineStr"/>
+      <c r="N214" t="inlineStr"/>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P214" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q214" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R214" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S214" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T214" t="inlineStr">
+        <is>
+          <t>3EB0EDF7499D737A99C175</t>
+        </is>
+      </c>
+      <c r="U214" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Moto Center</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Loja de peças para motocicletas</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>(99) 98218-9990</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>5599982189990</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr"/>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:32</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K215" t="inlineStr"/>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:32</t>
+        </is>
+      </c>
+      <c r="M215" t="inlineStr"/>
+      <c r="N215" t="inlineStr"/>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P215" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q215" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R215" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S215" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T215" t="inlineStr">
+        <is>
+          <t>3EB09391E2472F76075D73</t>
+        </is>
+      </c>
+      <c r="U215" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>MOTO PEÇAS REVISÃO</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Loja de motocicletas</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>(99) 99106-1317</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>5599991061317</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr"/>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:33</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K216" t="inlineStr"/>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:33</t>
+        </is>
+      </c>
+      <c r="M216" t="inlineStr"/>
+      <c r="N216" t="inlineStr"/>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P216" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q216" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R216" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S216" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T216" t="inlineStr">
+        <is>
+          <t>3EB0F11BD5A5139EA0419C</t>
+        </is>
+      </c>
+      <c r="U216" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Piu Motos Peças e Preparações</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Oficina mecânica</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>(99) 98480-7257</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>5599984807257</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr"/>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:35</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K217" t="inlineStr"/>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>18/05/2026 08:35</t>
+        </is>
+      </c>
+      <c r="M217" t="inlineStr"/>
+      <c r="N217" t="inlineStr"/>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P217" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q217" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R217" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S217" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T217" t="inlineStr">
+        <is>
+          <t>3EB0D9E6BEF56E48AD81C8</t>
+        </is>
+      </c>
+      <c r="U217" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Ferrari Moto Peças</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Oficina mecânica de motos</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>(99) 3541-5641</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>559935415641</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr"/>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:46</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K218" t="inlineStr"/>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:46</t>
+        </is>
+      </c>
+      <c r="M218" t="inlineStr"/>
+      <c r="N218" t="inlineStr"/>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P218" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q218" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R218" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S218" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T218" t="inlineStr">
+        <is>
+          <t>3EB0A20509F12D4134A96D</t>
+        </is>
+      </c>
+      <c r="U218" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>KSS MOTOS BALSAS</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Loja de peças para motocicletas</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>(99) 98480-8984</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>5599984808984</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr"/>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:47</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K219" t="inlineStr"/>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:47</t>
+        </is>
+      </c>
+      <c r="M219" t="inlineStr"/>
+      <c r="N219" t="inlineStr"/>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P219" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q219" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R219" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S219" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T219" t="inlineStr">
+        <is>
+          <t>3EB0DE09035B7F8BC05AB8</t>
+        </is>
+      </c>
+      <c r="U219" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>MF Motos</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Loja</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>(99) 3541-1446</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>559935411446</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr"/>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:49</t>
+        </is>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K220" t="inlineStr"/>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:49</t>
+        </is>
+      </c>
+      <c r="M220" t="inlineStr"/>
+      <c r="N220" t="inlineStr"/>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P220" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q220" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R220" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S220" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T220" t="inlineStr">
+        <is>
+          <t>D463C672ECE06BA66254</t>
+        </is>
+      </c>
+      <c r="U220" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Motoka Peças</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Oficina mecânica de motos</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>(99) 98818-5632</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>5599988185632</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr"/>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:50</t>
+        </is>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K221" t="inlineStr"/>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:50</t>
+        </is>
+      </c>
+      <c r="M221" t="inlineStr"/>
+      <c r="N221" t="inlineStr"/>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P221" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q221" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R221" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S221" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T221" t="inlineStr">
+        <is>
+          <t>3EB0479AFC8BB7D2BF3B6A</t>
+        </is>
+      </c>
+      <c r="U221" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Mix Moto Peças</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Loja de motocicletas</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>(99) 3541-9721</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>559935419721</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr"/>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:52</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K222" t="inlineStr"/>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:52</t>
+        </is>
+      </c>
+      <c r="M222" t="inlineStr"/>
+      <c r="N222" t="inlineStr"/>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P222" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q222" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R222" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S222" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T222" t="inlineStr">
+        <is>
+          <t>3EB0186F9620BDC4EE36C3</t>
+        </is>
+      </c>
+      <c r="U222" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Mc Motopeças</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Oficina mecânica de motos</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>(99) 3541-9246</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>559935419246</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr"/>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:53</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K223" t="inlineStr"/>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:53</t>
+        </is>
+      </c>
+      <c r="M223" t="inlineStr"/>
+      <c r="N223" t="inlineStr"/>
+      <c r="O223" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P223" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q223" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R223" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S223" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T223" t="inlineStr">
+        <is>
+          <t>3EB0DEBBA2848D17704804</t>
+        </is>
+      </c>
+      <c r="U223" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Universal Motos</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Oficina mecânica de motos</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>(99) 3541-6722</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>559935416722</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr"/>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:55</t>
+        </is>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K224" t="inlineStr"/>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:55</t>
+        </is>
+      </c>
+      <c r="M224" t="inlineStr"/>
+      <c r="N224" t="inlineStr"/>
+      <c r="O224" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P224" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q224" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R224" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S224" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T224" t="inlineStr">
+        <is>
+          <t>3EB0999496E4D8A013B1CC</t>
+        </is>
+      </c>
+      <c r="U224" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>SANTOS MOTO PEÇAS</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Loja</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>(99) 99902-0544</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>5599999020544</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr"/>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:56</t>
+        </is>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K225" t="inlineStr"/>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:56</t>
+        </is>
+      </c>
+      <c r="M225" t="inlineStr"/>
+      <c r="N225" t="inlineStr"/>
+      <c r="O225" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P225" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q225" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R225" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S225" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T225" t="inlineStr">
+        <is>
+          <t>3EB07193158BF45DC7DE3A</t>
+        </is>
+      </c>
+      <c r="U225" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>HF Moto Peças</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Oficina mecânica de motos</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>(99) 98826-4757</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>5599988264757</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr"/>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:58</t>
+        </is>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K226" t="inlineStr"/>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:58</t>
+        </is>
+      </c>
+      <c r="M226" t="inlineStr"/>
+      <c r="N226" t="inlineStr"/>
+      <c r="O226" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P226" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q226" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R226" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S226" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T226" t="inlineStr">
+        <is>
+          <t>3EB078375EDF0706EF84A1</t>
+        </is>
+      </c>
+      <c r="U226" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>R-A MOTO PEÇAS</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Loja de peças para motocicletas</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>(99) 98180-8079</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>5599981808079</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr"/>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:59</t>
+        </is>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K227" t="inlineStr"/>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>18/05/2026 10:59</t>
+        </is>
+      </c>
+      <c r="M227" t="inlineStr"/>
+      <c r="N227" t="inlineStr"/>
+      <c r="O227" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P227" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q227" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R227" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S227" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T227" t="inlineStr">
+        <is>
+          <t>3EB07668416F078DCBAF3B</t>
+        </is>
+      </c>
+      <c r="U227" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Rafael Moto Peças</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Oficina mecânica de motos</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>(99) 99651-3788</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>5599996513788</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr"/>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>18/05/2026 11:01</t>
+        </is>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K228" t="inlineStr"/>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>18/05/2026 11:01</t>
+        </is>
+      </c>
+      <c r="M228" t="inlineStr"/>
+      <c r="N228" t="inlineStr"/>
+      <c r="O228" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P228" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q228" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R228" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S228" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T228" t="inlineStr">
+        <is>
+          <t>3EB07287A8B18214059FB4</t>
+        </is>
+      </c>
+      <c r="U228" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Graúna Motos</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Concessionária Honda</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>(99) 3541-4618</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>559935414618</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr"/>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:28</t>
+        </is>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K229" t="inlineStr"/>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:28</t>
+        </is>
+      </c>
+      <c r="M229" t="inlineStr"/>
+      <c r="N229" t="inlineStr"/>
+      <c r="O229" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P229" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q229" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R229" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S229" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T229" t="inlineStr">
+        <is>
+          <t>94AAE6F199BB109B6D60</t>
+        </is>
+      </c>
+      <c r="U229" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>MOTOPLENA</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Loja de motocicletas</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>(99) 3541-3839</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>559935413839</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr"/>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:29</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K230" t="inlineStr"/>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:29</t>
+        </is>
+      </c>
+      <c r="M230" t="inlineStr"/>
+      <c r="N230" t="inlineStr"/>
+      <c r="O230" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P230" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q230" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R230" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S230" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T230" t="inlineStr">
+        <is>
+          <t>3EB0AC56DA05D8050FC113</t>
+        </is>
+      </c>
+      <c r="U230" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Soares Moto peças</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Oficina mecânica</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>(99) 98838-5327</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>5599988385327</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr"/>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:31</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K231" t="inlineStr"/>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:31</t>
+        </is>
+      </c>
+      <c r="M231" t="inlineStr"/>
+      <c r="N231" t="inlineStr"/>
+      <c r="O231" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P231" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q231" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R231" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S231" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T231" t="inlineStr">
+        <is>
+          <t>3EB0D0619D0AB3F34FD200</t>
+        </is>
+      </c>
+      <c r="U231" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Gilberto Moto Peças</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Oficina mecânica</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>(99) 99641-6975</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>5599996416975</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr"/>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:32</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K232" t="inlineStr"/>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:32</t>
+        </is>
+      </c>
+      <c r="M232" t="inlineStr"/>
+      <c r="N232" t="inlineStr"/>
+      <c r="O232" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P232" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q232" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R232" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S232" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T232" t="inlineStr">
+        <is>
+          <t>3EB06668AFD0A4A5D547C6</t>
+        </is>
+      </c>
+      <c r="U232" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Estilo Motos</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Oficina mecânica de motos</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>(99) 98112-7701</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>5599981127701</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr"/>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:34</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K233" t="inlineStr"/>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:34</t>
+        </is>
+      </c>
+      <c r="M233" t="inlineStr"/>
+      <c r="N233" t="inlineStr"/>
+      <c r="O233" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P233" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q233" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R233" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S233" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T233" t="inlineStr">
+        <is>
+          <t>3EB031CBCA24BAF2FB5461</t>
+        </is>
+      </c>
+      <c r="U233" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>WT MOTO PEÇAS</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Oficina mecânica de motos</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>(99) 99179-5139</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>5599991795139</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr"/>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:35</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K234" t="inlineStr"/>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:35</t>
+        </is>
+      </c>
+      <c r="M234" t="inlineStr"/>
+      <c r="N234" t="inlineStr"/>
+      <c r="O234" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P234" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q234" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R234" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S234" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T234" t="inlineStr">
+        <is>
+          <t>3EB0DF25015F1C757ED4F9</t>
+        </is>
+      </c>
+      <c r="U234" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>RS Moto peças</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Loja de peças para motocicletas</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>(99) 98404-6519</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>5599984046519</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr"/>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:37</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K235" t="inlineStr"/>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:37</t>
+        </is>
+      </c>
+      <c r="M235" t="inlineStr"/>
+      <c r="N235" t="inlineStr"/>
+      <c r="O235" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P235" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q235" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R235" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S235" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T235" t="inlineStr">
+        <is>
+          <t>3EB06458C1A9D64EE404DA</t>
+        </is>
+      </c>
+      <c r="U235" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Ernestino Motos</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Loja</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>(99) 98197-7822</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>5599981977822</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr"/>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:38</t>
+        </is>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K236" t="inlineStr"/>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:38</t>
+        </is>
+      </c>
+      <c r="M236" t="inlineStr"/>
+      <c r="N236" t="inlineStr"/>
+      <c r="O236" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P236" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q236" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R236" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S236" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T236" t="inlineStr">
+        <is>
+          <t>3EB0B93D7C0C1CEF45C73C</t>
+        </is>
+      </c>
+      <c r="U236" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Israel Motos</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Escritório da empresa</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>(99) 98453-2750</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>5599984532750</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr"/>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:40</t>
+        </is>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K237" t="inlineStr"/>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:40</t>
+        </is>
+      </c>
+      <c r="M237" t="inlineStr"/>
+      <c r="N237" t="inlineStr"/>
+      <c r="O237" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P237" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q237" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R237" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S237" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T237" t="inlineStr">
+        <is>
+          <t>3EB01FD81C2AE7E1890C4A</t>
+        </is>
+      </c>
+      <c r="U237" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Prestige Motos</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Loja de peças para motocicletas</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>(99) 98852-8310</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>5599988528310</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>BALSAS</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr"/>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:41</t>
+        </is>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K238" t="inlineStr"/>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:41</t>
+        </is>
+      </c>
+      <c r="M238" t="inlineStr"/>
+      <c r="N238" t="inlineStr"/>
+      <c r="O238" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P238" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q238" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R238" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S238" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T238" t="inlineStr">
+        <is>
+          <t>3EB0BFC7081F56C0FB8743</t>
+        </is>
+      </c>
+      <c r="U238" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>TKL MOTOS</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Oficina mecânica de motos</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>(99) 99197-5484</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>5599991975484</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr"/>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:43</t>
+        </is>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K239" t="inlineStr"/>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:43</t>
+        </is>
+      </c>
+      <c r="M239" t="inlineStr"/>
+      <c r="N239" t="inlineStr"/>
+      <c r="O239" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P239" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q239" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R239" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S239" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T239" t="inlineStr">
+        <is>
+          <t>3EB0739B0D96E1C5DCB98A</t>
+        </is>
+      </c>
+      <c r="U239" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Mega conserto de motos</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Oficina mecânica de motos</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>(99) 98508-3121</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>5599985083121</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr"/>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:44</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K240" t="inlineStr"/>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:44</t>
+        </is>
+      </c>
+      <c r="M240" t="inlineStr"/>
+      <c r="N240" t="inlineStr"/>
+      <c r="O240" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P240" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q240" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R240" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S240" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T240" t="inlineStr">
+        <is>
+          <t>3EB04407777A56DAEADC5D</t>
+        </is>
+      </c>
+      <c r="U240" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>PERFIL PEÇAS</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Loja de bicicleta</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>(99) 98180-5523</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>5599981805523</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr"/>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:46</t>
+        </is>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K241" t="inlineStr"/>
+      <c r="L241" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:46</t>
+        </is>
+      </c>
+      <c r="M241" t="inlineStr"/>
+      <c r="N241" t="inlineStr"/>
+      <c r="O241" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P241" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q241" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R241" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S241" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T241" t="inlineStr">
+        <is>
+          <t>3EB0CB290609C6A6E9F506</t>
+        </is>
+      </c>
+      <c r="U241" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Nenem motos</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Oficina mecânica</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>(99) 99145-9244</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>5599991459244</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr"/>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:47</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K242" t="inlineStr"/>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:47</t>
+        </is>
+      </c>
+      <c r="M242" t="inlineStr"/>
+      <c r="N242" t="inlineStr"/>
+      <c r="O242" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P242" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q242" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R242" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S242" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T242" t="inlineStr">
+        <is>
+          <t>3EB03BB47BFD28111D3CBA</t>
+        </is>
+      </c>
+      <c r="U242" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Tontoy Motos - Moto Peças - Oficina Amazonas</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Oficina mecânica</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>(33) 99802-7296</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>5533998027296</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr"/>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:49</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K243" t="inlineStr"/>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>19/05/2026 10:49</t>
+        </is>
+      </c>
+      <c r="M243" t="inlineStr"/>
+      <c r="N243" t="inlineStr"/>
+      <c r="O243" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P243" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q243" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R243" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S243" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T243" t="inlineStr">
+        <is>
+          <t>E761CEB7F383F04DA888</t>
+        </is>
+      </c>
+      <c r="U243" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Corrige integracao Sances e fallback de agendamento
</commit_message>
<xml_diff>
--- a/templates/data/disparo_atacado.xlsx
+++ b/templates/data/disparo_atacado.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U243"/>
+  <dimension ref="A1:U258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20757,6 +20757,1371 @@
         </is>
       </c>
     </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>M.W.M Moto Peças</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Oficina mecânica de motos</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>(99) 99151-1480</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>5599991511480</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr"/>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:12</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K244" t="inlineStr"/>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:12</t>
+        </is>
+      </c>
+      <c r="M244" t="inlineStr"/>
+      <c r="N244" t="inlineStr"/>
+      <c r="O244" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P244" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q244" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R244" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S244" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T244" t="inlineStr">
+        <is>
+          <t>3EB067B77CB41709424DEF</t>
+        </is>
+      </c>
+      <c r="U244" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Mundial Motos</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Loja de peças para motocicletas</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>(99) 98257-4335</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>5599982574335</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr"/>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:13</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K245" t="inlineStr"/>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:13</t>
+        </is>
+      </c>
+      <c r="M245" t="inlineStr"/>
+      <c r="N245" t="inlineStr"/>
+      <c r="O245" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P245" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q245" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R245" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S245" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T245" t="inlineStr">
+        <is>
+          <t>3EB0219CC47599B8A4CB9D</t>
+        </is>
+      </c>
+      <c r="U245" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>A+Moto</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Oficina mecânica de motos</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>(99) 98126-2557</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>5599981262557</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr"/>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:15</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K246" t="inlineStr"/>
+      <c r="L246" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:15</t>
+        </is>
+      </c>
+      <c r="M246" t="inlineStr"/>
+      <c r="N246" t="inlineStr"/>
+      <c r="O246" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P246" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q246" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R246" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S246" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T246" t="inlineStr">
+        <is>
+          <t>1990BDC50CBA8D42F726</t>
+        </is>
+      </c>
+      <c r="U246" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Comercial Motos 3 Irmãos</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Oficina mecânica de motos</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>(99) 98817-0045</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>5599988170045</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr"/>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:16</t>
+        </is>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K247" t="inlineStr"/>
+      <c r="L247" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:16</t>
+        </is>
+      </c>
+      <c r="M247" t="inlineStr"/>
+      <c r="N247" t="inlineStr"/>
+      <c r="O247" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P247" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q247" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R247" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S247" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T247" t="inlineStr">
+        <is>
+          <t>3EB08FBB091A58CAAB818C</t>
+        </is>
+      </c>
+      <c r="U247" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Rio motos</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Oficina mecânica de motos</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>(99) 3526-3448</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>559935263448</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr"/>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:18</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K248" t="inlineStr"/>
+      <c r="L248" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:18</t>
+        </is>
+      </c>
+      <c r="M248" t="inlineStr"/>
+      <c r="N248" t="inlineStr"/>
+      <c r="O248" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P248" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q248" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R248" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S248" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T248" t="inlineStr">
+        <is>
+          <t>3EB03A7130902C7665D3E7</t>
+        </is>
+      </c>
+      <c r="U248" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>JL MOTOS</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Mecânico</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>(99) 99174-7318</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>5599991747318</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr"/>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:19</t>
+        </is>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K249" t="inlineStr"/>
+      <c r="L249" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:19</t>
+        </is>
+      </c>
+      <c r="M249" t="inlineStr"/>
+      <c r="N249" t="inlineStr"/>
+      <c r="O249" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P249" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q249" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R249" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S249" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T249" t="inlineStr">
+        <is>
+          <t>3EB0A72F547FEE8CC2BD0C</t>
+        </is>
+      </c>
+      <c r="U249" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Honda Motoca</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Concessionária Honda</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>(99) 2101-0500</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>559921010500</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr"/>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:21</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K250" t="inlineStr"/>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:21</t>
+        </is>
+      </c>
+      <c r="M250" t="inlineStr"/>
+      <c r="N250" t="inlineStr"/>
+      <c r="O250" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P250" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q250" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R250" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S250" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T250" t="inlineStr">
+        <is>
+          <t>3EB0C4A798876519109302</t>
+        </is>
+      </c>
+      <c r="U250" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Chico Motopeças</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Loja de motocicletas</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>(99) 3524-7409</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>559935247409</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr"/>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:22</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K251" t="inlineStr"/>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:22</t>
+        </is>
+      </c>
+      <c r="M251" t="inlineStr"/>
+      <c r="N251" t="inlineStr"/>
+      <c r="O251" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P251" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q251" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R251" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S251" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T251" t="inlineStr">
+        <is>
+          <t>3EB0064C549ABF574D4E9C</t>
+        </is>
+      </c>
+      <c r="U251" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Moto Peças Menezes</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Loja de peças para motocicletas</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>(99) 98120-5421</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>5599981205421</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr"/>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:24</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K252" t="inlineStr"/>
+      <c r="L252" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:24</t>
+        </is>
+      </c>
+      <c r="M252" t="inlineStr"/>
+      <c r="N252" t="inlineStr"/>
+      <c r="O252" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P252" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q252" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R252" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S252" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T252" t="inlineStr">
+        <is>
+          <t>3EB09E298D1D50C5E808F8</t>
+        </is>
+      </c>
+      <c r="U252" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Casé Motos</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Loja</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>(63) 99259-6376</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>5563992596376</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr"/>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:25</t>
+        </is>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K253" t="inlineStr"/>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:25</t>
+        </is>
+      </c>
+      <c r="M253" t="inlineStr"/>
+      <c r="N253" t="inlineStr"/>
+      <c r="O253" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P253" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q253" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R253" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S253" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T253" t="inlineStr">
+        <is>
+          <t>3EB0B28310E5FB7A2CCA32</t>
+        </is>
+      </c>
+      <c r="U253" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Outfit Motos</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Loja de peças para motocicletas</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>(99) 99219-2337</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>5599992192337</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr"/>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:27</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K254" t="inlineStr"/>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:27</t>
+        </is>
+      </c>
+      <c r="M254" t="inlineStr"/>
+      <c r="N254" t="inlineStr"/>
+      <c r="O254" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P254" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q254" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R254" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S254" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T254" t="inlineStr">
+        <is>
+          <t>3EB049D86B18680C2A94BE</t>
+        </is>
+      </c>
+      <c r="U254" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Rossi Motors</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Oficina mecânica</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>(99) 98526-3909</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>5599985263909</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr"/>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:28</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K255" t="inlineStr"/>
+      <c r="L255" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:28</t>
+        </is>
+      </c>
+      <c r="M255" t="inlineStr"/>
+      <c r="N255" t="inlineStr"/>
+      <c r="O255" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P255" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q255" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R255" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S255" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T255" t="inlineStr">
+        <is>
+          <t>3EB0A67B6430BC596709A0</t>
+        </is>
+      </c>
+      <c r="U255" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Auto Peças Imperatriz</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Loja de autopeças</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>(99) 98257-0154</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>5599982570154</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr"/>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:30</t>
+        </is>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K256" t="inlineStr"/>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:30</t>
+        </is>
+      </c>
+      <c r="M256" t="inlineStr"/>
+      <c r="N256" t="inlineStr"/>
+      <c r="O256" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P256" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q256" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R256" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S256" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T256" t="inlineStr">
+        <is>
+          <t>3EB0D3451EB79FA0B4ED35</t>
+        </is>
+      </c>
+      <c r="U256" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Mottu Imperatriz</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Agência de aluguel de motocicletas</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>(11) 3181-8188</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>551131818188</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr"/>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:31</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K257" t="inlineStr"/>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:31</t>
+        </is>
+      </c>
+      <c r="M257" t="inlineStr"/>
+      <c r="N257" t="inlineStr"/>
+      <c r="O257" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P257" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q257" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R257" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S257" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T257" t="inlineStr">
+        <is>
+          <t>3EB06739715861CAB0447F</t>
+        </is>
+      </c>
+      <c r="U257" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Gr Motos</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Oficina mecânica de motos</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>(99) 99179-1295</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>5599991791295</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>IMPERATRIZ</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>ENVIADO</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr"/>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:33</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>AGUARDANDO</t>
+        </is>
+      </c>
+      <c r="K258" t="inlineStr"/>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>20/05/2026 08:33</t>
+        </is>
+      </c>
+      <c r="M258" t="inlineStr"/>
+      <c r="N258" t="inlineStr"/>
+      <c r="O258" t="inlineStr">
+        <is>
+          <t>Disparo atacado enviado com sucesso via botões Z-API</t>
+        </is>
+      </c>
+      <c r="P258" t="inlineStr">
+        <is>
+          <t>CAMPANHA_ATACADO_BOTOES</t>
+        </is>
+      </c>
+      <c r="Q258" t="inlineStr">
+        <is>
+          <t>atacado</t>
+        </is>
+      </c>
+      <c r="R258" t="inlineStr">
+        <is>
+          <t>AGUARDAR_RETORNO</t>
+        </is>
+      </c>
+      <c r="S258" t="inlineStr">
+        <is>
+          <t>MORNO</t>
+        </is>
+      </c>
+      <c r="T258" t="inlineStr">
+        <is>
+          <t>3EB07ECFF03F927674B6C3</t>
+        </is>
+      </c>
+      <c r="U258" t="inlineStr">
+        <is>
+          <t>BOTOES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>